<commit_message>
Add Duck Creek Sr. Services Project Manager application package
</commit_message>
<xml_diff>
--- a/applications/Job_Matches_Paris_ProductAI.xlsx
+++ b/applications/Job_Matches_Paris_ProductAI.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1370"/>
+  <dimension ref="A1:Q1370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -546,6 +546,26 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sent_date</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -61610,7 +61630,6 @@
       </c>
     </row>
     <row r="1348">
-      <c r="A1348" t="inlineStr"/>
       <c r="B1348" t="n">
         <v>5</v>
       </c>
@@ -61629,11 +61648,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1348" t="inlineStr"/>
-      <c r="G1348" t="inlineStr"/>
-      <c r="H1348" t="inlineStr"/>
-      <c r="I1348" t="inlineStr"/>
-      <c r="J1348" t="inlineStr"/>
       <c r="K1348" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/believe-91896.html</t>
@@ -61651,7 +61665,6 @@
       </c>
     </row>
     <row r="1349">
-      <c r="A1349" t="inlineStr"/>
       <c r="B1349" t="n">
         <v>5</v>
       </c>
@@ -61670,11 +61683,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1349" t="inlineStr"/>
-      <c r="G1349" t="inlineStr"/>
-      <c r="H1349" t="inlineStr"/>
-      <c r="I1349" t="inlineStr"/>
-      <c r="J1349" t="inlineStr"/>
       <c r="L1349" t="inlineStr">
         <is>
           <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
@@ -61687,7 +61695,6 @@
       </c>
     </row>
     <row r="1350">
-      <c r="A1350" t="inlineStr"/>
       <c r="B1350" t="n">
         <v>4</v>
       </c>
@@ -61706,11 +61713,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1350" t="inlineStr"/>
-      <c r="G1350" t="inlineStr"/>
-      <c r="H1350" t="inlineStr"/>
-      <c r="I1350" t="inlineStr"/>
-      <c r="J1350" t="inlineStr"/>
       <c r="K1350" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/alan-116878.html</t>
@@ -61728,7 +61730,6 @@
       </c>
     </row>
     <row r="1351">
-      <c r="A1351" t="inlineStr"/>
       <c r="B1351" t="n">
         <v>4</v>
       </c>
@@ -61747,11 +61748,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1351" t="inlineStr"/>
-      <c r="G1351" t="inlineStr"/>
-      <c r="H1351" t="inlineStr"/>
-      <c r="I1351" t="inlineStr"/>
-      <c r="J1351" t="inlineStr"/>
       <c r="L1351" t="inlineStr">
         <is>
           <t>Strength: AI relevance. Gap: no target-sector bonus.</t>
@@ -61764,7 +61760,6 @@
       </c>
     </row>
     <row r="1352">
-      <c r="A1352" t="inlineStr"/>
       <c r="B1352" t="n">
         <v>4</v>
       </c>
@@ -61783,11 +61778,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1352" t="inlineStr"/>
-      <c r="G1352" t="inlineStr"/>
-      <c r="H1352" t="inlineStr"/>
-      <c r="I1352" t="inlineStr"/>
-      <c r="J1352" t="inlineStr"/>
       <c r="L1352" t="inlineStr">
         <is>
           <t>Strength: AI relevance. Gap: no target-sector bonus.</t>
@@ -61800,7 +61790,6 @@
       </c>
     </row>
     <row r="1353">
-      <c r="A1353" t="inlineStr"/>
       <c r="B1353" t="n">
         <v>4</v>
       </c>
@@ -61819,11 +61808,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1353" t="inlineStr"/>
-      <c r="G1353" t="inlineStr"/>
-      <c r="H1353" t="inlineStr"/>
-      <c r="I1353" t="inlineStr"/>
-      <c r="J1353" t="inlineStr"/>
       <c r="L1353" t="inlineStr">
         <is>
           <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
@@ -61836,7 +61820,6 @@
       </c>
     </row>
     <row r="1354">
-      <c r="A1354" t="inlineStr"/>
       <c r="B1354" t="n">
         <v>4</v>
       </c>
@@ -61855,11 +61838,6 @@
           <t>Paris 13e - 75</t>
         </is>
       </c>
-      <c r="F1354" t="inlineStr"/>
-      <c r="G1354" t="inlineStr"/>
-      <c r="H1354" t="inlineStr"/>
-      <c r="I1354" t="inlineStr"/>
-      <c r="J1354" t="inlineStr"/>
       <c r="L1354" t="inlineStr">
         <is>
           <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
@@ -61872,7 +61850,6 @@
       </c>
     </row>
     <row r="1355">
-      <c r="A1355" t="inlineStr"/>
       <c r="B1355" t="n">
         <v>4</v>
       </c>
@@ -61891,11 +61868,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1355" t="inlineStr"/>
-      <c r="G1355" t="inlineStr"/>
-      <c r="H1355" t="inlineStr"/>
-      <c r="I1355" t="inlineStr"/>
-      <c r="J1355" t="inlineStr"/>
       <c r="K1355" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/contentsquare-97142.html</t>
@@ -61913,7 +61885,6 @@
       </c>
     </row>
     <row r="1356">
-      <c r="A1356" t="inlineStr"/>
       <c r="B1356" t="n">
         <v>4</v>
       </c>
@@ -61932,11 +61903,6 @@
           <t>Nanterre</t>
         </is>
       </c>
-      <c r="F1356" t="inlineStr"/>
-      <c r="G1356" t="inlineStr"/>
-      <c r="H1356" t="inlineStr"/>
-      <c r="I1356" t="inlineStr"/>
-      <c r="J1356" t="inlineStr"/>
       <c r="K1356" t="inlineStr">
         <is>
           <t>https://www.glassdoor.fr/job-listing/responsable-du-pôle-product-management-secteur-energie-fh-groupe-talents-handicap-JV_IC3019245_KO0,57_KE58,81.htm?jl=1010245287964</t>
@@ -61954,7 +61920,6 @@
       </c>
     </row>
     <row r="1357">
-      <c r="A1357" t="inlineStr"/>
       <c r="B1357" t="n">
         <v>3</v>
       </c>
@@ -61973,11 +61938,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1357" t="inlineStr"/>
-      <c r="G1357" t="inlineStr"/>
-      <c r="H1357" t="inlineStr"/>
-      <c r="I1357" t="inlineStr"/>
-      <c r="J1357" t="inlineStr"/>
       <c r="L1357" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -61990,7 +61950,6 @@
       </c>
     </row>
     <row r="1358">
-      <c r="A1358" t="inlineStr"/>
       <c r="B1358" t="n">
         <v>3</v>
       </c>
@@ -62009,11 +61968,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1358" t="inlineStr"/>
-      <c r="G1358" t="inlineStr"/>
-      <c r="H1358" t="inlineStr"/>
-      <c r="I1358" t="inlineStr"/>
-      <c r="J1358" t="inlineStr"/>
       <c r="K1358" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/front-107796.html</t>
@@ -62031,7 +61985,6 @@
       </c>
     </row>
     <row r="1359">
-      <c r="A1359" t="inlineStr"/>
       <c r="B1359" t="n">
         <v>3</v>
       </c>
@@ -62050,11 +62003,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1359" t="inlineStr"/>
-      <c r="G1359" t="inlineStr"/>
-      <c r="H1359" t="inlineStr"/>
-      <c r="I1359" t="inlineStr"/>
-      <c r="J1359" t="inlineStr"/>
       <c r="L1359" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62067,7 +62015,6 @@
       </c>
     </row>
     <row r="1360">
-      <c r="A1360" t="inlineStr"/>
       <c r="B1360" t="n">
         <v>3</v>
       </c>
@@ -62086,11 +62033,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1360" t="inlineStr"/>
-      <c r="G1360" t="inlineStr"/>
-      <c r="H1360" t="inlineStr"/>
-      <c r="I1360" t="inlineStr"/>
-      <c r="J1360" t="inlineStr"/>
       <c r="L1360" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62103,7 +62045,6 @@
       </c>
     </row>
     <row r="1361">
-      <c r="A1361" t="inlineStr"/>
       <c r="B1361" t="n">
         <v>2</v>
       </c>
@@ -62122,11 +62063,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1361" t="inlineStr"/>
-      <c r="G1361" t="inlineStr"/>
-      <c r="H1361" t="inlineStr"/>
-      <c r="I1361" t="inlineStr"/>
-      <c r="J1361" t="inlineStr"/>
       <c r="L1361" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62139,7 +62075,6 @@
       </c>
     </row>
     <row r="1362">
-      <c r="A1362" t="inlineStr"/>
       <c r="B1362" t="n">
         <v>2</v>
       </c>
@@ -62158,11 +62093,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1362" t="inlineStr"/>
-      <c r="G1362" t="inlineStr"/>
-      <c r="H1362" t="inlineStr"/>
-      <c r="I1362" t="inlineStr"/>
-      <c r="J1362" t="inlineStr"/>
       <c r="K1362" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/murex-108701.html</t>
@@ -62180,7 +62110,6 @@
       </c>
     </row>
     <row r="1363">
-      <c r="A1363" t="inlineStr"/>
       <c r="B1363" t="n">
         <v>2</v>
       </c>
@@ -62199,11 +62128,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1363" t="inlineStr"/>
-      <c r="G1363" t="inlineStr"/>
-      <c r="H1363" t="inlineStr"/>
-      <c r="I1363" t="inlineStr"/>
-      <c r="J1363" t="inlineStr"/>
       <c r="L1363" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62216,7 +62140,6 @@
       </c>
     </row>
     <row r="1364">
-      <c r="A1364" t="inlineStr"/>
       <c r="B1364" t="n">
         <v>2</v>
       </c>
@@ -62235,11 +62158,6 @@
           <t>Paris 7e - 75</t>
         </is>
       </c>
-      <c r="F1364" t="inlineStr"/>
-      <c r="G1364" t="inlineStr"/>
-      <c r="H1364" t="inlineStr"/>
-      <c r="I1364" t="inlineStr"/>
-      <c r="J1364" t="inlineStr"/>
       <c r="L1364" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62252,7 +62170,6 @@
       </c>
     </row>
     <row r="1365">
-      <c r="A1365" t="inlineStr"/>
       <c r="B1365" t="n">
         <v>1</v>
       </c>
@@ -62271,11 +62188,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1365" t="inlineStr"/>
-      <c r="G1365" t="inlineStr"/>
-      <c r="H1365" t="inlineStr"/>
-      <c r="I1365" t="inlineStr"/>
-      <c r="J1365" t="inlineStr"/>
       <c r="L1365" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62288,7 +62200,6 @@
       </c>
     </row>
     <row r="1366">
-      <c r="A1366" t="inlineStr"/>
       <c r="B1366" t="n">
         <v>1</v>
       </c>
@@ -62307,11 +62218,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1366" t="inlineStr"/>
-      <c r="G1366" t="inlineStr"/>
-      <c r="H1366" t="inlineStr"/>
-      <c r="I1366" t="inlineStr"/>
-      <c r="J1366" t="inlineStr"/>
       <c r="L1366" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62324,7 +62230,6 @@
       </c>
     </row>
     <row r="1367">
-      <c r="A1367" t="inlineStr"/>
       <c r="B1367" t="n">
         <v>1</v>
       </c>
@@ -62343,11 +62248,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1367" t="inlineStr"/>
-      <c r="G1367" t="inlineStr"/>
-      <c r="H1367" t="inlineStr"/>
-      <c r="I1367" t="inlineStr"/>
-      <c r="J1367" t="inlineStr"/>
       <c r="L1367" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62360,7 +62260,6 @@
       </c>
     </row>
     <row r="1368">
-      <c r="A1368" t="inlineStr"/>
       <c r="B1368" t="n">
         <v>1</v>
       </c>
@@ -62379,11 +62278,6 @@
           <t>Paris 7e - 75</t>
         </is>
       </c>
-      <c r="F1368" t="inlineStr"/>
-      <c r="G1368" t="inlineStr"/>
-      <c r="H1368" t="inlineStr"/>
-      <c r="I1368" t="inlineStr"/>
-      <c r="J1368" t="inlineStr"/>
       <c r="L1368" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62396,7 +62290,6 @@
       </c>
     </row>
     <row r="1369">
-      <c r="A1369" t="inlineStr"/>
       <c r="B1369" t="n">
         <v>0</v>
       </c>
@@ -62415,11 +62308,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1369" t="inlineStr"/>
-      <c r="G1369" t="inlineStr"/>
-      <c r="H1369" t="inlineStr"/>
-      <c r="I1369" t="inlineStr"/>
-      <c r="J1369" t="inlineStr"/>
       <c r="L1369" t="inlineStr">
         <is>
           <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
@@ -62432,7 +62320,6 @@
       </c>
     </row>
     <row r="1370">
-      <c r="A1370" t="inlineStr"/>
       <c r="B1370" t="n">
         <v>0</v>
       </c>
@@ -62451,11 +62338,6 @@
           <t>Paris - 75</t>
         </is>
       </c>
-      <c r="F1370" t="inlineStr"/>
-      <c r="G1370" t="inlineStr"/>
-      <c r="H1370" t="inlineStr"/>
-      <c r="I1370" t="inlineStr"/>
-      <c r="J1370" t="inlineStr"/>
       <c r="K1370" t="inlineStr">
         <is>
           <t>https://www.hellowork.com/fr-fr/entreprises/chanel-88659.html</t>

</xml_diff>

<commit_message>
CV Coach scan 2026-10-29
</commit_message>
<xml_diff>
--- a/applications/Job_Matches_Paris_ProductAI.xlsx
+++ b/applications/Job_Matches_Paris_ProductAI.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1370"/>
+  <dimension ref="A1:Q1387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -62354,6 +62354,907 @@
         </is>
       </c>
     </row>
+    <row r="1371">
+      <c r="A1371" t="n">
+        <v>1261</v>
+      </c>
+      <c r="B1371" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>VP, Technology Product Manager</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1371" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=VP%20Technology%20Product%20Manager%20BlackRock&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1371" t="inlineStr">
+        <is>
+          <t>BlackRock target-sector asset manager, VP seniority matches 15yr background; title doesn't name AI explicitly so ai_relevance partial. Biggest strength: target sector + seniority. Gap: no explicit AI/ML scope stated, no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1371" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="n">
+        <v>1262</v>
+      </c>
+      <c r="B1372" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>Head of Data Solution - F/H</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>AXA Partners</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>Malakoff (92)</t>
+        </is>
+      </c>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1372" t="inlineStr">
+        <is>
+          <t>https://fr.indeed.com/viewjob?jk=5dd5b932036ac801</t>
+        </is>
+      </c>
+      <c r="L1372" t="inlineStr">
+        <is>
+          <t>AXA target-sector insurer, Head-level data leadership overlaps data/AI strategy background. Biggest strength: target sector + seniority. Gap: AI relevance only implied by 'Data Solution', not explicit; no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1372" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="n">
+        <v>1263</v>
+      </c>
+      <c r="B1373" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - Financial Services Ops</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>Spendesk</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Paris (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1373" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Senior%20Product%20Manager%20Financial%20Services%20Ops%20Spendesk&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1373" t="inlineStr">
+        <is>
+          <t>Spendesk target-sector fintech, Senior level fits. Gap: no explicit AI relevance, no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1373" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="n">
+        <v>1264</v>
+      </c>
+      <c r="B1374" t="n">
+        <v>7</v>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Staff Product Manager - Loans</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>Qonto</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>Paris (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1374" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Staff%20Product%20Manager%20Loans%20Qonto&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1374" t="inlineStr">
+        <is>
+          <t>Qonto target-sector fintech, Staff level fits seniority. Gap: loans scope not explicitly AI-driven, no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1374" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="n">
+        <v>1265</v>
+      </c>
+      <c r="B1375" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Product Manager, Digital Assets - CSD &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>Euronext</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1375" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Product%20Manager%20Digital%20Assets%20CSD%20Settlement%20Euronext&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1375" t="inlineStr">
+        <is>
+          <t>Euronext target-sector financial infrastructure, strong domain match. Gap: no seniority qualifier (mid-level title), no AI relevance, no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1375" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="n">
+        <v>1266</v>
+      </c>
+      <c r="B1376" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>Head of Test Platform</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>Rothschild &amp; Co</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1376" t="inlineStr">
+        <is>
+          <t>https://fr.indeed.com/viewjob?jk=d22f27056931f624</t>
+        </is>
+      </c>
+      <c r="L1376" t="inlineStr">
+        <is>
+          <t>Large financial institution but role is test/QA platform leadership, not core product management. Gap: not a named target_sectors company, no AI relevance, no recruiter.</t>
+        </is>
+      </c>
+      <c r="M1376" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="n">
+        <v>1267</v>
+      </c>
+      <c r="B1377" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Manager Leader Produit Successions Contacts et demandes F/H</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>BPCE Solutions informatiques</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1377" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Manager%20Leader%20Produit%20Successions%20BPCE&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1377" t="inlineStr">
+        <is>
+          <t>BPCE target-sector bank, but mid-level ops/successions scope, no AI relevance.</t>
+        </is>
+      </c>
+      <c r="M1377" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="n">
+        <v>1268</v>
+      </c>
+      <c r="B1378" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Leader de Tribu - Marketing Digital (F/H)</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>Crédit Agricole Technologies et Services</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Paris (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1378" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Leader%20de%20Tribu%20Marketing%20Digital%20Credit%20Agricole&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1378" t="inlineStr">
+        <is>
+          <t>Crédit Agricole target-sector bank but marketing-digital tribe lead, not core product/AI role.</t>
+        </is>
+      </c>
+      <c r="M1378" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="n">
+        <v>1269</v>
+      </c>
+      <c r="B1379" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Product Owner - Intraday Continuous Market – Post-Trading Product</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>EPEX SPOT</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Paris (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1379" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=Product%20Owner%20Intraday%20Continuous%20Market%20EPEX%20SPOT&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1379" t="inlineStr">
+        <is>
+          <t>Energy trading markets post-trade domain overlap but not a named target sector, no AI relevance.</t>
+        </is>
+      </c>
+      <c r="M1379" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="n">
+        <v>1270</v>
+      </c>
+      <c r="B1380" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Product Manager - AI Platform H/F</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>Joko</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1380" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/82747414.html</t>
+        </is>
+      </c>
+      <c r="L1380" t="inlineStr">
+        <is>
+          <t>Cashback/fintech-adjacent app, explicit AI Platform scope, but not a named target company, mid-level title.</t>
+        </is>
+      </c>
+      <c r="M1380" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="n">
+        <v>1271</v>
+      </c>
+      <c r="B1381" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>Lead Product Manager - AI Platform H/F</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>Joko</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1381" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/83179274.html</t>
+        </is>
+      </c>
+      <c r="L1381" t="inlineStr">
+        <is>
+          <t>Same as above but Lead seniority bumps the score slightly; still not a named target sector.</t>
+        </is>
+      </c>
+      <c r="M1381" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="n">
+        <v>1272</v>
+      </c>
+      <c r="B1382" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>AI Platforms &amp; Agentic Solutions Product Manager F/H</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>Atos</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>Bezons</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1382" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/search/?keywords=AI%20Platforms%20Agentic%20Solutions%20Product%20Manager%20Atos&amp;location=Paris</t>
+        </is>
+      </c>
+      <c r="L1382" t="inlineStr">
+        <is>
+          <t>IT services company (not financial domain), explicit agentic-AI relevance, but not target sector, mid-level.</t>
+        </is>
+      </c>
+      <c r="M1382" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="n">
+        <v>1273</v>
+      </c>
+      <c r="B1383" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>Product Manager - AI Inference H/F</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>Scaleway</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1383" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/84913129.html</t>
+        </is>
+      </c>
+      <c r="L1383" t="inlineStr">
+        <is>
+          <t>AI infra cloud company, explicit AI relevance, but no financial domain overlap, not target sector.</t>
+        </is>
+      </c>
+      <c r="M1383" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="n">
+        <v>1274</v>
+      </c>
+      <c r="B1384" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Head Of Product Data H/F</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>Scaleway</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1384" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/84442744.html</t>
+        </is>
+      </c>
+      <c r="L1384" t="inlineStr">
+        <is>
+          <t>Head-level data leadership but AI infra company, no financial-domain overlap, not target sector.</t>
+        </is>
+      </c>
+      <c r="M1384" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="n">
+        <v>1275</v>
+      </c>
+      <c r="B1385" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>XDR Product Owner</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>AXA</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1385" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.fr/job-listing/xdr-product-owner-axa-singapore-JV_IC2881970_KO0,17_KE18,31.htm</t>
+        </is>
+      </c>
+      <c r="L1385" t="inlineStr">
+        <is>
+          <t>AXA target-sector insurer, but cybersecurity (XDR) Product Owner role — domain is financial but functional fit (security vs AI/product strategy) is weak, mid-level title.</t>
+        </is>
+      </c>
+      <c r="M1385" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="n">
+        <v>1276</v>
+      </c>
+      <c r="B1386" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Data Product Manager H/F</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>Hymaïa</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1386" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/82079025.html</t>
+        </is>
+      </c>
+      <c r="L1386" t="inlineStr">
+        <is>
+          <t>Small consultancy-adjacent data company, not target sector, no explicit AI or seniority signal.</t>
+        </is>
+      </c>
+      <c r="M1386" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="n">
+        <v>1277</v>
+      </c>
+      <c r="B1387" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Senior Product Manager Orienté·e Data &amp; ai H/F</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>AlumnForce</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="K1387" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/emplois/83469970.html</t>
+        </is>
+      </c>
+      <c r="L1387" t="inlineStr">
+        <is>
+          <t>EdTech/alumni platform, Senior level and explicit AI mention give some credit but no financial-domain overlap, not target sector.</t>
+        </is>
+      </c>
+      <c r="M1387" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>